<commit_message>
perbaharuan struktur dan perubahan kecil alur kpi
</commit_message>
<xml_diff>
--- a/public/template_KPI/template_import_kpi.xlsx
+++ b/public/template_KPI/template_import_kpi.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\INIXINDO\Documents\vicky\INIXCOFFEE\public\template_KPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B25AB25-E709-4603-8DB1-3F33DC8246FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A2A347-DAB5-46E8-A934-58BF6F1DB953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
     <author>System</author>
   </authors>
   <commentList>
-    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="C2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -39,7 +39,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="95">
   <si>
     <t>judul_kpi</t>
   </si>
@@ -72,18 +72,9 @@
     <t>karyawan</t>
   </si>
   <si>
-    <t>jangka_target</t>
-  </si>
-  <si>
     <t>detail_jangka</t>
   </si>
   <si>
-    <t>tipe_target</t>
-  </si>
-  <si>
-    <t>nilai_target</t>
-  </si>
-  <si>
     <t>asistant_route</t>
   </si>
   <si>
@@ -97,12 +88,6 @@
   </si>
   <si>
     <t>Budi Santoso, Siti Aminah</t>
-  </si>
-  <si>
-    <t>Tahunan</t>
-  </si>
-  <si>
-    <t>2024</t>
   </si>
   <si>
     <t>Tabel Referensi Assistant Route</t>
@@ -397,7 +382,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -420,12 +405,6 @@
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor rgb="FF4F46E5"/>
       </patternFill>
     </fill>
   </fills>
@@ -475,9 +454,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -783,15 +760,13 @@
   <dimension ref="A1:Q1340"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="19" customWidth="1"/>
-    <col min="5" max="5" width="27" customWidth="1"/>
-    <col min="6" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="4" max="4" width="27" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="19" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
     <col min="13" max="13" width="10.5703125" style="3" customWidth="1"/>
     <col min="14" max="14" width="17.85546875" style="5" customWidth="1"/>
@@ -801,95 +776,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="13"/>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
       <c r="N1" s="12" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O1" s="12"/>
       <c r="P1" s="12"/>
       <c r="Q1" s="12"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
       <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2">
+        <v>2024</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="10"/>
+      <c r="N2" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="P2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q2" s="7" t="s">
         <v>11</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>63</v>
-      </c>
-      <c r="I2" s="10">
-        <v>80000000000</v>
-      </c>
-      <c r="J2" t="s">
-        <v>17</v>
-      </c>
-      <c r="N2" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="O2" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="P2" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q2" s="7" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I3" s="10"/>
       <c r="N3" s="11" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="O3" s="11" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -897,10 +857,10 @@
       <c r="N4" s="11"/>
       <c r="O4" s="11"/>
       <c r="P4" s="3" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="Q4" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -908,10 +868,10 @@
       <c r="N5" s="11"/>
       <c r="O5" s="11"/>
       <c r="P5" s="4" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="Q5" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -919,17 +879,17 @@
       <c r="N6" s="11"/>
       <c r="O6" s="11"/>
       <c r="P6" s="3" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I7" s="10"/>
       <c r="N7" s="11"/>
       <c r="O7" s="11" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -937,7 +897,7 @@
       <c r="N8" s="11"/>
       <c r="O8" s="11"/>
       <c r="P8" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
@@ -945,17 +905,17 @@
       <c r="N9" s="11"/>
       <c r="O9" s="11"/>
       <c r="P9" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I10" s="10"/>
       <c r="N10" s="11"/>
       <c r="O10" s="11" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
@@ -963,7 +923,7 @@
       <c r="N11" s="11"/>
       <c r="O11" s="11"/>
       <c r="P11" s="3" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
@@ -971,7 +931,7 @@
       <c r="N12" s="11"/>
       <c r="O12" s="11"/>
       <c r="P12" s="4" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
@@ -979,17 +939,17 @@
       <c r="N13" s="11"/>
       <c r="O13" s="11"/>
       <c r="P13" s="4" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="I14" s="10"/>
       <c r="N14" s="11"/>
       <c r="O14" s="11" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="P14" s="3" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
@@ -997,7 +957,7 @@
       <c r="N15" s="11"/>
       <c r="O15" s="11"/>
       <c r="P15" s="3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
@@ -1005,17 +965,17 @@
       <c r="N16" s="11"/>
       <c r="O16" s="11"/>
       <c r="P16" s="4" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I17" s="10"/>
       <c r="N17" s="11"/>
       <c r="O17" s="11" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="9:16" x14ac:dyDescent="0.25">
@@ -1023,7 +983,7 @@
       <c r="N18" s="11"/>
       <c r="O18" s="11"/>
       <c r="P18" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="9:16" x14ac:dyDescent="0.25">
@@ -1031,7 +991,7 @@
       <c r="N19" s="11"/>
       <c r="O19" s="11"/>
       <c r="P19" s="4" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="9:16" x14ac:dyDescent="0.25">
@@ -1039,17 +999,17 @@
       <c r="N20" s="11"/>
       <c r="O20" s="11"/>
       <c r="P20" s="4" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I21" s="10"/>
       <c r="N21" s="11"/>
       <c r="O21" s="11" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="P21" s="4" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="9:16" x14ac:dyDescent="0.25">
@@ -1057,17 +1017,17 @@
       <c r="N22" s="11"/>
       <c r="O22" s="11"/>
       <c r="P22" s="4" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I23" s="10"/>
       <c r="N23" s="11"/>
       <c r="O23" s="11" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="P23" s="4" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="9:16" x14ac:dyDescent="0.25">
@@ -1075,7 +1035,7 @@
       <c r="N24" s="11"/>
       <c r="O24" s="11"/>
       <c r="P24" s="4" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="9:16" x14ac:dyDescent="0.25">
@@ -1083,17 +1043,17 @@
       <c r="N25" s="11"/>
       <c r="O25" s="11"/>
       <c r="P25" s="4" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I26" s="10"/>
       <c r="N26" s="11"/>
       <c r="O26" s="11" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="P26" s="4" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="9:16" x14ac:dyDescent="0.25">
@@ -1101,27 +1061,27 @@
       <c r="N27" s="11"/>
       <c r="O27" s="11"/>
       <c r="P27" s="4" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I28" s="10"/>
       <c r="N28" s="11"/>
       <c r="O28" s="5" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="P28" s="4" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="29" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I29" s="10"/>
       <c r="N29" s="11"/>
       <c r="O29" s="11" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="P29" s="4" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30" spans="9:16" x14ac:dyDescent="0.25">
@@ -1129,17 +1089,17 @@
       <c r="N30" s="11"/>
       <c r="O30" s="11"/>
       <c r="P30" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I31" s="10"/>
       <c r="N31" s="11"/>
       <c r="O31" s="11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="P31" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="32" spans="9:16" x14ac:dyDescent="0.25">
@@ -1147,7 +1107,7 @@
       <c r="N32" s="11"/>
       <c r="O32" s="11"/>
       <c r="P32" s="4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33" spans="9:16" x14ac:dyDescent="0.25">
@@ -1155,17 +1115,17 @@
       <c r="N33" s="11"/>
       <c r="O33" s="11"/>
       <c r="P33" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="34" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I34" s="10"/>
       <c r="N34" s="11"/>
       <c r="O34" s="11" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="P34" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="35" spans="9:16" x14ac:dyDescent="0.25">
@@ -1173,17 +1133,17 @@
       <c r="N35" s="11"/>
       <c r="O35" s="11"/>
       <c r="P35" s="4" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I36" s="10"/>
       <c r="N36" s="11"/>
       <c r="O36" s="11" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="P36" s="4" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37" spans="9:16" x14ac:dyDescent="0.25">
@@ -1191,17 +1151,17 @@
       <c r="N37" s="11"/>
       <c r="O37" s="11"/>
       <c r="P37" s="4" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="38" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I38" s="10"/>
       <c r="N38" s="11"/>
       <c r="O38" s="11" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="P38" s="4" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="39" spans="9:16" x14ac:dyDescent="0.25">
@@ -1209,17 +1169,17 @@
       <c r="N39" s="11"/>
       <c r="O39" s="11"/>
       <c r="P39" s="4" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="40" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I40" s="10"/>
       <c r="N40" s="11"/>
       <c r="O40" s="11" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="P40" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="41" spans="9:16" x14ac:dyDescent="0.25">
@@ -1227,7 +1187,7 @@
       <c r="N41" s="11"/>
       <c r="O41" s="11"/>
       <c r="P41" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="42" spans="9:16" x14ac:dyDescent="0.25">
@@ -1235,17 +1195,17 @@
       <c r="N42" s="11"/>
       <c r="O42" s="11"/>
       <c r="P42" s="4" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="43" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I43" s="10"/>
       <c r="N43" s="11"/>
       <c r="O43" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="P43" s="4" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" spans="9:16" x14ac:dyDescent="0.25">
@@ -1253,71 +1213,71 @@
       <c r="N44" s="11"/>
       <c r="O44" s="11"/>
       <c r="P44" s="4" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I45" s="10"/>
       <c r="N45" s="11"/>
       <c r="O45" s="5" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="P45" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="46" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I46" s="10"/>
       <c r="N46" s="11"/>
       <c r="O46" s="5" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="P46" s="4" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
     <row r="47" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I47" s="10"/>
       <c r="N47" s="11" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="O47" s="9" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="P47" s="4" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="48" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I48" s="10"/>
       <c r="N48" s="11"/>
       <c r="O48" s="5" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="P48" s="4" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="49" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I49" s="10"/>
       <c r="N49" s="11" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="O49" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="P49" s="4" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="50" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I50" s="10"/>
       <c r="N50" s="11"/>
       <c r="O50" s="11" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="P50" s="4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="51" spans="9:16" x14ac:dyDescent="0.25">
@@ -1325,7 +1285,7 @@
       <c r="N51" s="11"/>
       <c r="O51" s="11"/>
       <c r="P51" s="4" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="52" spans="9:16" x14ac:dyDescent="0.25">
@@ -1333,27 +1293,27 @@
       <c r="N52" s="11"/>
       <c r="O52" s="11"/>
       <c r="P52" s="4" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="53" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I53" s="10"/>
       <c r="N53" s="11"/>
       <c r="O53" s="5" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="P53" s="4" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="54" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I54" s="10"/>
       <c r="N54" s="11"/>
       <c r="O54" s="11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="P54" s="4" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="55" spans="9:16" x14ac:dyDescent="0.25">
@@ -1361,17 +1321,17 @@
       <c r="N55" s="11"/>
       <c r="O55" s="11"/>
       <c r="P55" s="4" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="56" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I56" s="10"/>
       <c r="N56" s="11"/>
       <c r="O56" s="11" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="P56" s="4" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="57" spans="9:16" x14ac:dyDescent="0.25">
@@ -1379,17 +1339,17 @@
       <c r="N57" s="11"/>
       <c r="O57" s="11"/>
       <c r="P57" s="4" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="58" spans="9:16" x14ac:dyDescent="0.25">
       <c r="I58" s="10"/>
       <c r="N58" s="11"/>
       <c r="O58" s="5" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="P58" s="4" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="59" spans="9:16" x14ac:dyDescent="0.25">
@@ -5263,12 +5223,9 @@
     <mergeCell ref="O14:O16"/>
     <mergeCell ref="O17:O20"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1646" xr:uid="{5A2039C0-02E0-402B-9590-D294B6C152D3}">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1646" xr:uid="{5A2039C0-02E0-402B-9590-D294B6C152D3}">
       <formula1>$P$3:$P$58</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1030" xr:uid="{AC5D5014-6B36-451D-89D7-57B85AF602AD}">
-      <formula1>$Q$3:$Q$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>